<commit_message>
feat: chạy song song 2 cửa sổ quét + 1 cửa sổ bình luận, nhắm khách tìm màn hình ở Hà Nội
- Cửa sổ QUÉT (main.py quet [n], 2 cửa sổ chia nhóm qua bảng scan_claims) đưa bài đạt lọc vào hàng chờ;
  cửa sổ BÌNH LUẬN lấy bài mới nhất ra bình luận ngay (modules/scanner.py, modules/queue_runner.py)
- Xếp lịch quét theo hiệu quả nhóm: nhóm tương tác cao 2 phút, nhóm có khách 5 phút, nhóm kém 24 giờ
- Chuỗi bộ lọc bài: chủ đề (chỉ Màn hình) → ý định MUA/BÁN (từ khóa + Gemini) → khu vực (data/khu_vuc.txt)
  → tương tác; bỏ bài cũ hơn 6 giờ, tối đa 40 bài/ngày
- Nhóm Hà Nội chỉ cần từ 500 thành viên (nhóm toàn quốc giữ 5.000)
- Đăng bài theo lịch: bỏ qua nhóm chưa tham gia / không xem được / chỉ cho bán / giới hạn bài chờ duyệt
- Chrome: tắt DNS-over-HTTPS để hết lỗi ERR_NAME_NOT_RESOLVED khi chạy 3 Chrome
- Thêm 144 bài kiểm tra (pytest)
- Không đưa lên git nữa: CSDL (có SĐT), nhật ký bình luận, ảnh chụp bài viết — chỉ giữ trên máy chạy bot
</commit_message>
<xml_diff>
--- a/data/groups_found.xlsx
+++ b/data/groups_found.xlsx
@@ -1847,12 +1847,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/nghienbuildpc/</t>
+          <t>https://www.facebook.com/groups/fbccibd/</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nghiện Build PC</t>
+          <t>Mua Bán Màn Hình Máy Tính Cũ Việt Nam | Mua Bán &amp; Sửa Chữa</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>màn hình, mua bán màn hình</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1876,33 +1876,29 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>127000</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>3 bài viết/ngày</t>
-        </is>
-      </c>
+        <v>226000</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>PC Hà Nội</t>
+          <t>mua bán màn hình Hà Nội</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-04 22:59</t>
+          <t>2026-10-09 23:09</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/TinyPC/</t>
+          <t>https://www.facebook.com/groups/danbacu8386/</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tiny PC</t>
+          <t>Chợ PC - Linh Kiện Máy Tính</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1926,21 +1922,21 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>81000</v>
+        <v>204000</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>80+ bài viết/ngày</t>
+          <t>30+ bài viết/ngày</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>PC Hà Nội</t>
+          <t>màn hình Hà Nội</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-04 22:59</t>
+          <t>2026-10-06 21:42</t>
         </is>
       </c>
     </row>

</xml_diff>